<commit_message>
Added jobs 24 Jul 26
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC6B980C-39B4-4BE3-8F34-BA123B9E0C23}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE054966-D54A-4DC6-83D2-F0B6A500A3BF}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="396">
   <si>
     <t>Job</t>
   </si>
@@ -1176,6 +1176,57 @@
   </si>
   <si>
     <t>1084710 - 233751 - DG Label</t>
+  </si>
+  <si>
+    <t>37 Fry Road, Halcombe</t>
+  </si>
+  <si>
+    <t>1084770 - 00055238 - DG Label</t>
+  </si>
+  <si>
+    <t>338E Leedstown Road, Hunterville</t>
+  </si>
+  <si>
+    <t>1084772 - 00060405 - DG Label</t>
+  </si>
+  <si>
+    <t>9A Belvedere Crescent, Takaro</t>
+  </si>
+  <si>
+    <t>1084774 - 00053598 - DG Label</t>
+  </si>
+  <si>
+    <t>7 Long Melford Road, Awapuni</t>
+  </si>
+  <si>
+    <t>1084776 - 00045583 - DG Label</t>
+  </si>
+  <si>
+    <t>115 Atawhai Road, Fitzherbert</t>
+  </si>
+  <si>
+    <t>1084778 - 00045588 - DG Label</t>
+  </si>
+  <si>
+    <t>0000044918CP6D0</t>
+  </si>
+  <si>
+    <t>74 Cambridge Avenue, Ashhurst</t>
+  </si>
+  <si>
+    <t>1084779 - 00048369 - DG Label</t>
+  </si>
+  <si>
+    <t>75 Somerset Road, Springvale</t>
+  </si>
+  <si>
+    <t>1084780 - 00050330 - DG Label</t>
+  </si>
+  <si>
+    <t>5 Pukeko Place, Riversdale Beach</t>
+  </si>
+  <si>
+    <t>1084781 - 00059954 - DG Label</t>
   </si>
 </sst>
 </file>
@@ -1556,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C189"/>
+  <dimension ref="A1:C197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -3643,6 +3694,94 @@
         <v>327</v>
       </c>
     </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>395</v>
+      </c>
+      <c r="B190" t="s">
+        <v>394</v>
+      </c>
+      <c r="C190" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>393</v>
+      </c>
+      <c r="B191" t="s">
+        <v>392</v>
+      </c>
+      <c r="C191" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>391</v>
+      </c>
+      <c r="B192" t="s">
+        <v>390</v>
+      </c>
+      <c r="C192" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>388</v>
+      </c>
+      <c r="B193" t="s">
+        <v>387</v>
+      </c>
+      <c r="C193" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>386</v>
+      </c>
+      <c r="B194" t="s">
+        <v>385</v>
+      </c>
+      <c r="C194" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>384</v>
+      </c>
+      <c r="B195" t="s">
+        <v>383</v>
+      </c>
+      <c r="C195" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>382</v>
+      </c>
+      <c r="B196" t="s">
+        <v>381</v>
+      </c>
+      <c r="C196" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>380</v>
+      </c>
+      <c r="B197" t="s">
+        <v>379</v>
+      </c>
+      <c r="C197" t="s">
+        <v>327</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new job 24/7/26
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE054966-D54A-4DC6-83D2-F0B6A500A3BF}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CED83A92-01AD-456D-B8A3-C2FA243C4A99}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="395">
   <si>
     <t>Job</t>
   </si>
@@ -1206,9 +1206,6 @@
   </si>
   <si>
     <t>1084778 - 00045588 - DG Label</t>
-  </si>
-  <si>
-    <t>0000044918CP6D0</t>
   </si>
   <si>
     <t>74 Cambridge Avenue, Ashhurst</t>
@@ -3696,10 +3693,10 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B190" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C190" t="s">
         <v>327</v>
@@ -3707,10 +3704,10 @@
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B191" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C191" t="s">
         <v>326</v>
@@ -3718,13 +3715,13 @@
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B192" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C192" t="s">
-        <v>389</v>
+        <v>326</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -3784,5 +3781,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>